<commit_message>
Update dry-run contact workbook snapshot
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BfXsy4DaUQM1Riuguc26b
</commit_message>
<xml_diff>
--- a/enrich/EF_Start_contacts_dry_run.xlsx
+++ b/enrich/EF_Start_contacts_dry_run.xlsx
@@ -4926,7 +4926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4947,9 +4947,8 @@
           <t>Total contacts</t>
         </is>
       </c>
-      <c r="B3" s="2">
-        <f>COUNTA(Contacts!A2:A140)</f>
-        <v/>
+      <c r="B3" s="2" t="n">
+        <v>139</v>
       </c>
     </row>
     <row r="4">
@@ -4958,9 +4957,8 @@
           <t>With LinkedIn URL</t>
         </is>
       </c>
-      <c r="B4" s="2">
-        <f>COUNTIF(Contacts!D2:D140,"http*")</f>
-        <v/>
+      <c r="B4" s="2" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -4969,9 +4967,8 @@
           <t>With email</t>
         </is>
       </c>
-      <c r="B5" s="2">
-        <f>COUNTIF(Contacts!F2:F140,"?*")</f>
-        <v/>
+      <c r="B5" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -4980,9 +4977,8 @@
           <t>Without email</t>
         </is>
       </c>
-      <c r="B6" s="2">
-        <f>COUNTA(Contacts!A2:A140)-COUNTIF(Contacts!F2:F140,"?*")</f>
-        <v/>
+      <c r="B6" s="2" t="n">
+        <v>139</v>
       </c>
     </row>
     <row r="7">
@@ -4991,9 +4987,8 @@
           <t>With phone</t>
         </is>
       </c>
-      <c r="B7" s="2">
-        <f>COUNTIF(Contacts!H2:H140,"?*")</f>
-        <v/>
+      <c r="B7" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -5019,13 +5014,11 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B10" s="2">
-        <f>COUNTIF(Contacts!E2:E140,"*A*")</f>
-        <v/>
-      </c>
-      <c r="C10" s="2">
-        <f>COUNTIFS(Contacts!E2:E140,"*A*",Contacts!F2:F140,"?*")</f>
-        <v/>
+      <c r="B10" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -5034,13 +5027,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B11" s="2">
-        <f>COUNTIF(Contacts!E2:E140,"*B*")</f>
-        <v/>
-      </c>
-      <c r="C11" s="2">
-        <f>COUNTIFS(Contacts!E2:E140,"*B*",Contacts!F2:F140,"?*")</f>
-        <v/>
+      <c r="B11" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -5049,13 +5040,11 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B12" s="2">
-        <f>COUNTIF(Contacts!E2:E140,"*C*")</f>
-        <v/>
-      </c>
-      <c r="C12" s="2">
-        <f>COUNTIFS(Contacts!E2:E140,"*C*",Contacts!F2:F140,"?*")</f>
-        <v/>
+      <c r="B12" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -5064,13 +5053,11 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B13" s="2">
-        <f>COUNTIF(Contacts!E2:E140,"*D*")</f>
-        <v/>
-      </c>
-      <c r="C13" s="2">
-        <f>COUNTIFS(Contacts!E2:E140,"*D*",Contacts!F2:F140,"?*")</f>
-        <v/>
+      <c r="B13" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -5098,6 +5085,13 @@
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Email Confidence: high = verified VALID, medium = catch-all domain, low = unverified/risky.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Summary counts are a snapshot computed when this file was generated (2026-09-29).</t>
         </is>
       </c>
     </row>

</xml_diff>